<commit_message>
Attempted to test the fixes
</commit_message>
<xml_diff>
--- a/rules/CORE-001080/negative/01/data/unit-test-coreid-CG0288-negative 1.xlsx
+++ b/rules/CORE-001080/negative/01/data/unit-test-coreid-CG0288-negative 1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\verisian\core-contributor\rules\CORE-001080\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04B8130B-ADDB-496E-8149-A90C6552AC52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C1B9A42-A020-402D-8327-989ABFDA75BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="858" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="191">
   <si>
     <t>Product</t>
   </si>
@@ -176,9 +176,6 @@
     <t>Added on to Existing Treatments</t>
   </si>
   <si>
-    <t>C00001</t>
-  </si>
-  <si>
     <t>AGEMAX</t>
   </si>
   <si>
@@ -293,9 +290,6 @@
     <t>C00002</t>
   </si>
   <si>
-    <t>CDISC CT</t>
-  </si>
-  <si>
     <t>INDIC</t>
   </si>
   <si>
@@ -617,7 +611,7 @@
     <t>Record</t>
   </si>
   <si>
-    <t>sdtmct-2025-03-28</t>
+    <t>TEST</t>
   </si>
 </sst>
 </file>
@@ -702,7 +696,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -716,17 +710,8 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1145,18 +1130,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1174,27 +1159,27 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" style="10"/>
+    <col min="6" max="6" width="9.140625" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="7" t="s">
         <v>188</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1205,7 +1190,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D2">
         <v>7</v>
@@ -1213,8 +1198,8 @@
       <c r="E2" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="10" t="s">
-        <v>45</v>
+      <c r="F2" s="8" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1225,7 +1210,7 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D3">
         <v>7</v>
@@ -1233,7 +1218,7 @@
       <c r="E3" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="8" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1245,7 +1230,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D4">
         <v>7</v>
@@ -1253,8 +1238,8 @@
       <c r="E4" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="10" t="s">
-        <v>192</v>
+      <c r="F4" s="8" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1265,7 +1250,7 @@
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D5">
         <v>20</v>
@@ -1273,8 +1258,8 @@
       <c r="E5" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="10" t="s">
-        <v>83</v>
+      <c r="F5" s="8" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1285,7 +1270,7 @@
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D6">
         <v>20</v>
@@ -1293,8 +1278,8 @@
       <c r="E6" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="10" t="s">
-        <v>81</v>
+      <c r="F6" s="8" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1305,7 +1290,7 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D7">
         <v>20</v>
@@ -1313,8 +1298,8 @@
       <c r="E7" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="10" t="s">
-        <v>192</v>
+      <c r="F7" s="8" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1539,9 +1524,9 @@
         <v>39</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J7" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="J7" s="2" t="s">
         <v>41</v>
       </c>
       <c r="K7" s="4" t="s">
@@ -1559,13 +1544,13 @@
         <v>1</v>
       </c>
       <c r="E8" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -1579,16 +1564,16 @@
         <v>1</v>
       </c>
       <c r="E9" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="J9" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -1602,16 +1587,16 @@
         <v>1</v>
       </c>
       <c r="D10" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -1625,19 +1610,19 @@
         <v>1</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E11" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="G11" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="J11" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -1651,16 +1636,16 @@
         <v>1</v>
       </c>
       <c r="D12" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -1674,16 +1659,16 @@
         <v>2</v>
       </c>
       <c r="D13" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -1697,16 +1682,16 @@
         <v>3</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E14" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>62</v>
-      </c>
       <c r="G14" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -1720,16 +1705,16 @@
         <v>4</v>
       </c>
       <c r="D15" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -1743,13 +1728,13 @@
         <v>1</v>
       </c>
       <c r="E16" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="G16" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>70</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>40</v>
@@ -1772,13 +1757,13 @@
         <v>1</v>
       </c>
       <c r="E17" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="G17" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>73</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>40</v>
@@ -1801,13 +1786,13 @@
         <v>1</v>
       </c>
       <c r="E18" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F18" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="G18" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>40</v>
@@ -1830,19 +1815,19 @@
         <v>1</v>
       </c>
       <c r="E19" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="G19" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="I19" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="J19" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -1856,19 +1841,19 @@
         <v>1</v>
       </c>
       <c r="E20" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>82</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>39</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="J20" s="11" t="s">
-        <v>84</v>
+        <v>82</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>41</v>
       </c>
       <c r="K20" s="4" t="s">
         <v>42</v>
@@ -1885,22 +1870,22 @@
         <v>1</v>
       </c>
       <c r="E21" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="G21" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="I21" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="J21" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I21" s="2" t="s">
+      <c r="K21" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -1914,13 +1899,13 @@
         <v>1</v>
       </c>
       <c r="E22" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>40</v>
@@ -1943,13 +1928,13 @@
         <v>1</v>
       </c>
       <c r="E23" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G23" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>96</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>40</v>
@@ -1972,16 +1957,16 @@
         <v>1</v>
       </c>
       <c r="E24" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="F24" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>99</v>
-      </c>
       <c r="J24" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -1995,13 +1980,13 @@
         <v>1</v>
       </c>
       <c r="E25" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="G25" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="45" x14ac:dyDescent="0.25">
@@ -2015,16 +2000,16 @@
         <v>1</v>
       </c>
       <c r="D26" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="G26" s="2" t="s">
         <v>104</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="45" x14ac:dyDescent="0.25">
@@ -2038,16 +2023,16 @@
         <v>2</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -2061,13 +2046,13 @@
         <v>1</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="165" x14ac:dyDescent="0.25">
@@ -2081,16 +2066,16 @@
         <v>2</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E29" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G29" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="150" x14ac:dyDescent="0.25">
@@ -2104,16 +2089,16 @@
         <v>3</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F30" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G30" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="45" x14ac:dyDescent="0.25">
@@ -2127,16 +2112,16 @@
         <v>4</v>
       </c>
       <c r="D31" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="E31" s="2" t="s">
-        <v>109</v>
-      </c>
       <c r="F31" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="45" x14ac:dyDescent="0.25">
@@ -2150,16 +2135,16 @@
         <v>5</v>
       </c>
       <c r="D32" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="E32" s="2" t="s">
-        <v>109</v>
-      </c>
       <c r="F32" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -2173,19 +2158,19 @@
         <v>1</v>
       </c>
       <c r="E33" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G33" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="F33" s="2" t="s">
+      <c r="I33" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="G33" s="2" t="s">
+      <c r="J33" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="I33" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="J33" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -2199,13 +2184,13 @@
         <v>1</v>
       </c>
       <c r="E34" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="G34" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -2219,16 +2204,16 @@
         <v>1</v>
       </c>
       <c r="E35" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G35" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="I35" s="2" t="s">
         <v>124</v>
-      </c>
-      <c r="G35" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="I35" s="2" t="s">
-        <v>126</v>
       </c>
       <c r="J35" s="2" t="s">
         <v>41</v>
@@ -2248,13 +2233,13 @@
         <v>1</v>
       </c>
       <c r="E36" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G36" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="G36" s="2" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
@@ -2268,19 +2253,19 @@
         <v>1</v>
       </c>
       <c r="E37" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="G37" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="F37" s="2" t="s">
+      <c r="I37" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="J37" s="2" t="s">
         <v>131</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="I37" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="J37" s="2" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -2294,16 +2279,16 @@
         <v>1</v>
       </c>
       <c r="E38" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G38" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="F38" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>136</v>
-      </c>
       <c r="I38" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J38" s="2" t="s">
         <v>41</v>
@@ -2323,13 +2308,13 @@
         <v>1</v>
       </c>
       <c r="E39" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="G39" s="2" t="s">
         <v>137</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
@@ -2343,13 +2328,13 @@
         <v>1</v>
       </c>
       <c r="E40" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="G40" s="2" t="s">
         <v>140</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
@@ -2363,16 +2348,16 @@
         <v>1</v>
       </c>
       <c r="E41" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="G41" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F41" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="G41" s="2" t="s">
-        <v>145</v>
-      </c>
       <c r="J41" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
@@ -2386,16 +2371,16 @@
         <v>1</v>
       </c>
       <c r="E42" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="G42" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="F42" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>148</v>
-      </c>
       <c r="I42" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J42" s="2" t="s">
         <v>41</v>
@@ -2415,13 +2400,13 @@
         <v>1</v>
       </c>
       <c r="E43" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="G43" s="2" t="s">
         <v>149</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="G43" s="2" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
@@ -2435,16 +2420,16 @@
         <v>1</v>
       </c>
       <c r="E44" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="G44" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F44" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>154</v>
-      </c>
       <c r="J44" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
@@ -2458,13 +2443,13 @@
         <v>1</v>
       </c>
       <c r="E45" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G45" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
@@ -2478,16 +2463,16 @@
         <v>1</v>
       </c>
       <c r="E46" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G46" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="F46" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>160</v>
-      </c>
       <c r="I46" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J46" s="2" t="s">
         <v>41</v>
@@ -2507,16 +2492,16 @@
         <v>1</v>
       </c>
       <c r="E47" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="G47" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F47" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="G47" s="2" t="s">
-        <v>163</v>
-      </c>
       <c r="I47" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J47" s="2" t="s">
         <v>41</v>
@@ -2536,16 +2521,16 @@
         <v>1</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J48" s="2" t="s">
         <v>41</v>
@@ -2565,13 +2550,13 @@
         <v>1</v>
       </c>
       <c r="E49" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="G49" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="G49" s="2" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
@@ -2585,16 +2570,16 @@
         <v>1</v>
       </c>
       <c r="E50" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="G50" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="F50" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="G50" s="2" t="s">
-        <v>171</v>
-      </c>
       <c r="I50" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J50" s="2" t="s">
         <v>41</v>
@@ -2614,13 +2599,13 @@
         <v>1</v>
       </c>
       <c r="E51" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="G51" s="2" t="s">
         <v>172</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="G51" s="2" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -2634,16 +2619,16 @@
         <v>1</v>
       </c>
       <c r="E52" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="G52" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="F52" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="G52" s="2" t="s">
-        <v>177</v>
-      </c>
       <c r="I52" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J52" s="2" t="s">
         <v>41</v>
@@ -2663,19 +2648,19 @@
         <v>1</v>
       </c>
       <c r="E53" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="G53" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="F53" s="2" t="s">
+      <c r="I53" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="G53" s="2" t="s">
+      <c r="J53" s="2" t="s">
         <v>180</v>
-      </c>
-      <c r="I53" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="J53" s="2" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
@@ -2689,16 +2674,16 @@
         <v>1</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J54" s="2" t="s">
         <v>41</v>
@@ -2718,16 +2703,16 @@
         <v>2</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J55" s="2" t="s">
         <v>41</v>
@@ -2750,25 +2735,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Comment xmlns="9dee18c2-6da5-44c1-913e-bf7f393fe0e8" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010090ADB40D834AE945B19FCDA4041AC0CB" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d36826f407302d9fd93d8089214679b0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="9dee18c2-6da5-44c1-913e-bf7f393fe0e8" xmlns:ns3="63ea592b-d684-45c7-8cdc-fad8f8e6bb41" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="257daeb82d9c284d9d656fb5e9ad601e" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3008,26 +2974,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F04EB3C1-E279-4752-95AF-A2254F34364B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9dee18c2-6da5-44c1-913e-bf7f393fe0e8"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF9BEA20-DCD2-4199-AEB6-4F95B371C878}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Comment xmlns="9dee18c2-6da5-44c1-913e-bf7f393fe0e8" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90113CEE-35A4-4503-9D90-53C6490D5D89}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3045,4 +3011,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF9BEA20-DCD2-4199-AEB6-4F95B371C878}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F04EB3C1-E279-4752-95AF-A2254F34364B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9dee18c2-6da5-44c1-913e-bf7f393fe0e8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
adjusted to address feedback
</commit_message>
<xml_diff>
--- a/rules/CORE-001080/negative/01/data/unit-test-coreid-CG0288-negative 1.xlsx
+++ b/rules/CORE-001080/negative/01/data/unit-test-coreid-CG0288-negative 1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\verisian\core-contributor\rules\CORE-001080\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{225E1517-6691-4A97-91FD-16A4C7CB7E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E59474F-926C-4677-9FB5-A6F62218CB5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="858" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="361" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="91" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="197">
   <si>
     <t>Product</t>
   </si>
@@ -612,6 +612,24 @@
   </si>
   <si>
     <t>C00001</t>
+  </si>
+  <si>
+    <t>CDISC CT</t>
+  </si>
+  <si>
+    <t>RACEC</t>
+  </si>
+  <si>
+    <t>Race As Collected</t>
+  </si>
+  <si>
+    <t>YEMENI</t>
+  </si>
+  <si>
+    <t>C205490</t>
+  </si>
+  <si>
+    <t>2024-09-27</t>
   </si>
 </sst>
 </file>
@@ -1095,7 +1113,7 @@
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -1155,7 +1173,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECB89C6A-C749-457C-B0C8-0262E8FA0779}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
@@ -1244,7 +1262,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
@@ -1253,13 +1271,13 @@
         <v>189</v>
       </c>
       <c r="D5">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="E5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>82</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1276,10 +1294,10 @@
         <v>20</v>
       </c>
       <c r="E6" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1296,10 +1314,50 @@
         <v>20</v>
       </c>
       <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>189</v>
+      </c>
+      <c r="D8">
+        <v>20</v>
+      </c>
+      <c r="E8" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F8" s="8" t="s">
         <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>189</v>
+      </c>
+      <c r="D9">
+        <v>20</v>
+      </c>
+      <c r="E9" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -1526,7 +1584,7 @@
       <c r="I7" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="J7" s="4" t="s">
         <v>41</v>
       </c>
       <c r="K7" s="4" t="s">
@@ -1852,8 +1910,8 @@
       <c r="I20" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="J20" s="2" t="s">
-        <v>41</v>
+      <c r="J20" s="4" t="s">
+        <v>191</v>
       </c>
       <c r="K20" s="4" t="s">
         <v>42</v>
@@ -2703,22 +2761,22 @@
         <v>2</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>101</v>
+        <v>194</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>124</v>
+        <v>195</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>41</v>
+        <v>191</v>
       </c>
       <c r="K55" s="2" t="s">
-        <v>42</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added missing error data into validation sheet
</commit_message>
<xml_diff>
--- a/rules/CORE-001080/negative/01/data/unit-test-coreid-CG0288-negative 1.xlsx
+++ b/rules/CORE-001080/negative/01/data/unit-test-coreid-CG0288-negative 1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10920"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\verisian\core-contributor\rules\CORE-001080\negative\01\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/CORE-001080/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E59474F-926C-4677-9FB5-A6F62218CB5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE6F7137-EF50-9846-94DE-E57DE7AA39A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="361" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-7000" windowWidth="51200" windowHeight="28800" tabRatio="361" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="91" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="197">
   <si>
     <t>Product</t>
   </si>
@@ -1111,12 +1111,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43053ECA-A0F8-4801-9CFA-FD5472AA5759}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1124,7 +1124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1140,14 +1140,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="3.7109375" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1155,7 +1155,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -1173,14 +1173,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECB89C6A-C749-457C-B0C8-0262E8FA0779}">
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" style="8"/>
+    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.1640625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>183</v>
       </c>
@@ -1200,7 +1200,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1220,7 +1220,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1240,7 +1240,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1</v>
       </c>
@@ -1260,7 +1260,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1</v>
       </c>
@@ -1280,7 +1280,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2</v>
       </c>
@@ -1300,7 +1300,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2</v>
       </c>
@@ -1320,7 +1320,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2</v>
       </c>
@@ -1340,7 +1340,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2</v>
       </c>
@@ -1357,6 +1357,86 @@
         <v>17</v>
       </c>
       <c r="F9" s="8" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>189</v>
+      </c>
+      <c r="D10">
+        <v>55</v>
+      </c>
+      <c r="E10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" t="s">
+        <v>189</v>
+      </c>
+      <c r="D11">
+        <v>55</v>
+      </c>
+      <c r="E11" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>189</v>
+      </c>
+      <c r="D12">
+        <v>55</v>
+      </c>
+      <c r="E12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" t="s">
+        <v>189</v>
+      </c>
+      <c r="D13">
+        <v>55</v>
+      </c>
+      <c r="E13" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" s="8" t="s">
         <v>191</v>
       </c>
     </row>
@@ -1368,12 +1448,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F57D753-4466-4FD4-8C1D-984014BD1694}">
   <dimension ref="A1:K55"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="11" width="20.7109375" style="2" customWidth="1"/>
+    <col min="1" max="11" width="20.6640625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
@@ -1408,7 +1488,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>19</v>
       </c>
@@ -1443,7 +1523,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -1478,7 +1558,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>12</v>
       </c>
@@ -1513,7 +1593,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>32</v>
       </c>
@@ -1533,7 +1613,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>32</v>
       </c>
@@ -1562,7 +1642,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>32</v>
       </c>
@@ -1591,7 +1671,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>32</v>
       </c>
@@ -1611,7 +1691,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>32</v>
       </c>
@@ -1634,7 +1714,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>32</v>
       </c>
@@ -1657,7 +1737,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>32</v>
       </c>
@@ -1683,7 +1763,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>32</v>
       </c>
@@ -1706,7 +1786,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>32</v>
       </c>
@@ -1729,7 +1809,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>32</v>
       </c>
@@ -1752,7 +1832,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>32</v>
       </c>
@@ -1775,7 +1855,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>32</v>
       </c>
@@ -1804,7 +1884,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>32</v>
       </c>
@@ -1833,7 +1913,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>32</v>
       </c>
@@ -1862,7 +1942,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>32</v>
       </c>
@@ -1888,7 +1968,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>32</v>
       </c>
@@ -1917,7 +1997,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>32</v>
       </c>
@@ -1946,7 +2026,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>32</v>
       </c>
@@ -1975,7 +2055,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>32</v>
       </c>
@@ -2004,7 +2084,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>32</v>
       </c>
@@ -2027,7 +2107,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>32</v>
       </c>
@@ -2047,7 +2127,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>32</v>
       </c>
@@ -2070,7 +2150,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>32</v>
       </c>
@@ -2093,7 +2173,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>32</v>
       </c>
@@ -2113,7 +2193,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="165" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" ht="144" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>32</v>
       </c>
@@ -2136,7 +2216,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="150" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="128" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>32</v>
       </c>
@@ -2159,7 +2239,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>32</v>
       </c>
@@ -2182,7 +2262,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>32</v>
       </c>
@@ -2205,7 +2285,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>32</v>
       </c>
@@ -2231,7 +2311,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>32</v>
       </c>
@@ -2251,7 +2331,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>32</v>
       </c>
@@ -2280,7 +2360,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>32</v>
       </c>
@@ -2300,7 +2380,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>32</v>
       </c>
@@ -2326,7 +2406,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>32</v>
       </c>
@@ -2355,7 +2435,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>32</v>
       </c>
@@ -2375,7 +2455,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>32</v>
       </c>
@@ -2395,7 +2475,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>32</v>
       </c>
@@ -2418,7 +2498,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>32</v>
       </c>
@@ -2447,7 +2527,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>32</v>
       </c>
@@ -2467,7 +2547,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>32</v>
       </c>
@@ -2490,7 +2570,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>32</v>
       </c>
@@ -2510,7 +2590,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>32</v>
       </c>
@@ -2539,7 +2619,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>32</v>
       </c>
@@ -2568,7 +2648,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>32</v>
       </c>
@@ -2597,7 +2677,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>32</v>
       </c>
@@ -2617,7 +2697,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>32</v>
       </c>
@@ -2646,7 +2726,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
         <v>32</v>
       </c>
@@ -2666,7 +2746,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>32</v>
       </c>
@@ -2695,7 +2775,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
         <v>32</v>
       </c>
@@ -2721,7 +2801,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>32</v>
       </c>
@@ -2750,7 +2830,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>32</v>
       </c>
@@ -2760,7 +2840,7 @@
       <c r="C55" s="2">
         <v>2</v>
       </c>
-      <c r="E55" s="2" t="s">
+      <c r="E55" s="4" t="s">
         <v>192</v>
       </c>
       <c r="F55" s="2" t="s">
@@ -2769,13 +2849,13 @@
       <c r="G55" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="I55" s="2" t="s">
+      <c r="I55" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="J55" s="2" t="s">
+      <c r="J55" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="K55" s="2" t="s">
+      <c r="K55" s="4" t="s">
         <v>196</v>
       </c>
     </row>
@@ -2793,6 +2873,25 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Comment xmlns="9dee18c2-6da5-44c1-913e-bf7f393fe0e8" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010090ADB40D834AE945B19FCDA4041AC0CB" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d36826f407302d9fd93d8089214679b0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="9dee18c2-6da5-44c1-913e-bf7f393fe0e8" xmlns:ns3="63ea592b-d684-45c7-8cdc-fad8f8e6bb41" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="257daeb82d9c284d9d656fb5e9ad601e" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3032,26 +3131,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F04EB3C1-E279-4752-95AF-A2254F34364B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9dee18c2-6da5-44c1-913e-bf7f393fe0e8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Comment xmlns="9dee18c2-6da5-44c1-913e-bf7f393fe0e8" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF9BEA20-DCD2-4199-AEB6-4F95B371C878}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90113CEE-35A4-4503-9D90-53C6490D5D89}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3069,23 +3168,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF9BEA20-DCD2-4199-AEB6-4F95B371C878}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F04EB3C1-E279-4752-95AF-A2254F34364B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9dee18c2-6da5-44c1-913e-bf7f393fe0e8"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>